<commit_message>
README-Update: Neuer Screenshot, Rechtschreibfehler
Und neue Beispiel-XLSX.
</commit_message>
<xml_diff>
--- a/Beispiele/Ergebnisse.xlsx
+++ b/Beispiele/Ergebnisse.xlsx
@@ -7,23 +7,25 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Nebendepot US0846707026" sheetId="1" r:id="rId1"/>
-    <sheet name="Nebendepot IE00B3RBWM25" sheetId="2" r:id="rId2"/>
-    <sheet name="Nebendepot IE00BK5BQT80" sheetId="3" r:id="rId3"/>
-    <sheet name="Nebendepot FR0010755611" sheetId="4" r:id="rId4"/>
-    <sheet name="Hauptdepot IE00BK5BQT80" sheetId="5" r:id="rId5"/>
-    <sheet name="Hauptdepot IE00B3RBWM25" sheetId="6" r:id="rId6"/>
-    <sheet name="Hauptdepot US0378331005" sheetId="7" r:id="rId7"/>
-    <sheet name="Hauptdepot US0846707026" sheetId="8" r:id="rId8"/>
-    <sheet name="Hauptdepot DE0006231004" sheetId="9" r:id="rId9"/>
-    <sheet name="Hauptdepot FR0010755611" sheetId="10" r:id="rId10"/>
+    <sheet name="Übersicht" sheetId="1" r:id="rId1"/>
+    <sheet name="VAP" sheetId="2" r:id="rId2"/>
+    <sheet name="Nebendepot US0846707026" sheetId="3" r:id="rId3"/>
+    <sheet name="Nebendepot IE00B3RBWM25" sheetId="4" r:id="rId4"/>
+    <sheet name="Nebendepot IE00BK5BQT80" sheetId="5" r:id="rId5"/>
+    <sheet name="Nebendepot FR0010755611" sheetId="6" r:id="rId6"/>
+    <sheet name="Hauptdepot IE00BK5BQT80" sheetId="7" r:id="rId7"/>
+    <sheet name="Hauptdepot IE00B3RBWM25" sheetId="8" r:id="rId8"/>
+    <sheet name="Hauptdepot US0378331005" sheetId="9" r:id="rId9"/>
+    <sheet name="Hauptdepot US0846707026" sheetId="10" r:id="rId10"/>
+    <sheet name="Hauptdepot DE0006231004" sheetId="11" r:id="rId11"/>
+    <sheet name="Hauptdepot FR0010755611" sheetId="12" r:id="rId12"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="44">
   <si>
     <t>ISIN</t>
   </si>
@@ -31,6 +33,96 @@
     <t>Name</t>
   </si>
   <si>
+    <t>Depot</t>
+  </si>
+  <si>
+    <t>Brutto-Wert</t>
+  </si>
+  <si>
+    <t>KESt-pflichtiger Gewinn</t>
+  </si>
+  <si>
+    <t>KESt + Soli</t>
+  </si>
+  <si>
+    <t>Netto-Wert</t>
+  </si>
+  <si>
+    <t>Steueranteil an Brutto-Auszahlung</t>
+  </si>
+  <si>
+    <t>DE0006231004</t>
+  </si>
+  <si>
+    <t>FR0010755611</t>
+  </si>
+  <si>
+    <t>IE00B3RBWM25</t>
+  </si>
+  <si>
+    <t>IE00BK5BQT80</t>
+  </si>
+  <si>
+    <t>US0378331005</t>
+  </si>
+  <si>
+    <t>US0846707026</t>
+  </si>
+  <si>
+    <t>Summe</t>
+  </si>
+  <si>
+    <t>GESAMTSUMME</t>
+  </si>
+  <si>
+    <t>Infineon Technologies AG</t>
+  </si>
+  <si>
+    <t>Amundi Lev 2x MSCI USA Daily Acc ETF</t>
+  </si>
+  <si>
+    <t>Vanguard FTSE All-World Dist ETF</t>
+  </si>
+  <si>
+    <t>Vanguard FTSE All-World Acc ETF</t>
+  </si>
+  <si>
+    <t>Apple Inc.</t>
+  </si>
+  <si>
+    <t>Berkshire Hathaway B (BRK-B)</t>
+  </si>
+  <si>
+    <t>Hauptdepot</t>
+  </si>
+  <si>
+    <t>Nebendepot</t>
+  </si>
+  <si>
+    <t>2023 vor TFS</t>
+  </si>
+  <si>
+    <t>2023 nach TFS</t>
+  </si>
+  <si>
+    <t>2024 vor TFS</t>
+  </si>
+  <si>
+    <t>2024 nach TFS</t>
+  </si>
+  <si>
+    <t>2025 vor TFS</t>
+  </si>
+  <si>
+    <t>2025 nach TFS</t>
+  </si>
+  <si>
+    <t>Summe vor TFS</t>
+  </si>
+  <si>
+    <t>Summe nach TFS</t>
+  </si>
+  <si>
     <t>Datum Kauf</t>
   </si>
   <si>
@@ -46,27 +138,6 @@
     <t>Kosten pro Anteil</t>
   </si>
   <si>
-    <t>Brutto-Wert</t>
-  </si>
-  <si>
-    <t>KESt-pflichtiger Gewinn</t>
-  </si>
-  <si>
-    <t>KESt + Soli</t>
-  </si>
-  <si>
-    <t>Netto-Wert</t>
-  </si>
-  <si>
-    <t>Steueranteil an Brutto-Auszahlung</t>
-  </si>
-  <si>
-    <t>US0846707026</t>
-  </si>
-  <si>
-    <t>Berkshire Hathaway B (BRK-B)</t>
-  </si>
-  <si>
     <t>VAP 2025 vor TFS pro Anteil</t>
   </si>
   <si>
@@ -79,40 +150,13 @@
     <t>KESt-pflichtiger Gewinn nach VAP nach TFS</t>
   </si>
   <si>
-    <t>IE00B3RBWM25</t>
-  </si>
-  <si>
-    <t>Vanguard FTSE All-World Dist ETF</t>
-  </si>
-  <si>
     <t>VAP 2023 vor TFS pro Anteil</t>
   </si>
   <si>
     <t>VAP 2024 vor TFS pro Anteil</t>
   </si>
   <si>
-    <t>IE00BK5BQT80</t>
-  </si>
-  <si>
-    <t>Vanguard FTSE All-World Acc ETF</t>
-  </si>
-  <si>
-    <t>FR0010755611</t>
-  </si>
-  <si>
-    <t>Amundi Lev 2x MSCI USA Daily Acc ETF</t>
-  </si>
-  <si>
-    <t>US0378331005</t>
-  </si>
-  <si>
-    <t>Apple Inc.</t>
-  </si>
-  <si>
-    <t>DE0006231004</t>
-  </si>
-  <si>
-    <t>Infineon Technologies AG</t>
+    <t>KESt-pflichtiger Gewinn nach TFS</t>
   </si>
 </sst>
 </file>
@@ -467,6 +511,375 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H16"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="14.28515625" customWidth="1"/>
+    <col min="2" max="2" width="38.28515625" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="4" max="7" width="15.7109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="15.7109375" style="2" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="50" customHeight="1">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="1">
+        <v>860.1</v>
+      </c>
+      <c r="E2" s="1">
+        <v>507.7000000000001</v>
+      </c>
+      <c r="F2" s="1">
+        <v>133.905875</v>
+      </c>
+      <c r="G2" s="1">
+        <v>726.194125</v>
+      </c>
+      <c r="H2" s="2">
+        <v>0.155686402743867</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" s="1">
+        <v>617.1</v>
+      </c>
+      <c r="E3" s="1">
+        <v>65.37999999999997</v>
+      </c>
+      <c r="F3" s="1">
+        <v>17.24397499999999</v>
+      </c>
+      <c r="G3" s="1">
+        <v>599.856025</v>
+      </c>
+      <c r="H3" s="2">
+        <v>0.02794356668287148</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="1">
+        <v>5457</v>
+      </c>
+      <c r="E4" s="1">
+        <v>1097.225444306833</v>
+      </c>
+      <c r="F4" s="1">
+        <v>289.3932109359273</v>
+      </c>
+      <c r="G4" s="1">
+        <v>5167.606789064073</v>
+      </c>
+      <c r="H4" s="2">
+        <v>0.05303155780390825</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="1">
+        <v>12557.76</v>
+      </c>
+      <c r="E5" s="1">
+        <v>3308.772292297831</v>
+      </c>
+      <c r="F5" s="1">
+        <v>872.6886920935528</v>
+      </c>
+      <c r="G5" s="1">
+        <v>11685.07130790645</v>
+      </c>
+      <c r="H5" s="2">
+        <v>0.06949397759580951</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="1">
+        <v>6574.365000000001</v>
+      </c>
+      <c r="E6" s="1">
+        <v>3285.499174757282</v>
+      </c>
+      <c r="F6" s="1">
+        <v>866.550407342233</v>
+      </c>
+      <c r="G6" s="1">
+        <v>5707.814592657768</v>
+      </c>
+      <c r="H6" s="2">
+        <v>0.1318074684539469</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="1">
+        <v>2029.598921733715</v>
+      </c>
+      <c r="E7" s="1">
+        <v>1058.138564590858</v>
+      </c>
+      <c r="F7" s="1">
+        <v>279.0840464108387</v>
+      </c>
+      <c r="G7" s="1">
+        <v>1750.514875322876</v>
+      </c>
+      <c r="H7" s="2">
+        <v>0.1375069938312939</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="1">
+        <v>28095.92392173372</v>
+      </c>
+      <c r="E8" s="1">
+        <v>9322.715475952804</v>
+      </c>
+      <c r="F8" s="1">
+        <v>2458.866206782552</v>
+      </c>
+      <c r="G8" s="1">
+        <v>25637.05771495116</v>
+      </c>
+      <c r="H8" s="2">
+        <v>0.08751683032856185</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="1">
+        <v>3548.325</v>
+      </c>
+      <c r="E10" s="1">
+        <v>1093.968735157083</v>
+      </c>
+      <c r="F10" s="1">
+        <v>288.5342538976807</v>
+      </c>
+      <c r="G10" s="1">
+        <v>3259.79074610232</v>
+      </c>
+      <c r="H10" s="2">
+        <v>0.08131562184909238</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="1">
+        <v>21346.5</v>
+      </c>
+      <c r="E11" s="1">
+        <v>7099.086096402999</v>
+      </c>
+      <c r="F11" s="1">
+        <v>1872.383957926291</v>
+      </c>
+      <c r="G11" s="1">
+        <v>19474.11604207371</v>
+      </c>
+      <c r="H11" s="2">
+        <v>0.08771386212851244</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="1">
+        <v>824</v>
+      </c>
+      <c r="E12" s="1">
+        <v>281.649919775</v>
+      </c>
+      <c r="F12" s="1">
+        <v>74.28516634065625</v>
+      </c>
+      <c r="G12" s="1">
+        <v>749.7148336593438</v>
+      </c>
+      <c r="H12" s="2">
+        <v>0.09015190089885466</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D13" s="1">
+        <v>5317.549174942333</v>
+      </c>
+      <c r="E13" s="1">
+        <v>1093.106674942333</v>
+      </c>
+      <c r="F13" s="1">
+        <v>288.3068855160404</v>
+      </c>
+      <c r="G13" s="1">
+        <v>5029.242289426293</v>
+      </c>
+      <c r="H13" s="2">
+        <v>0.05421800081786117</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D14" s="1">
+        <v>31036.37417494234</v>
+      </c>
+      <c r="E14" s="1">
+        <v>9567.811426277416</v>
+      </c>
+      <c r="F14" s="1">
+        <v>2523.510263680668</v>
+      </c>
+      <c r="G14" s="1">
+        <v>28512.86391126167</v>
+      </c>
+      <c r="H14" s="2">
+        <v>0.08130815311918944</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="D16" s="1">
+        <v>59132.29809667604</v>
+      </c>
+      <c r="E16" s="1">
+        <v>18890.52690223022</v>
+      </c>
+      <c r="F16" s="1">
+        <v>4982.376470463219</v>
+      </c>
+      <c r="G16" s="1">
+        <v>54149.92162621283</v>
+      </c>
+      <c r="H16" s="2">
+        <v>0.08425812340858929</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -486,148 +899,148 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
+      <c r="J1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="K1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="C2" s="4">
-        <v>44382</v>
+        <v>43501</v>
       </c>
       <c r="D2">
-        <v>1.8</v>
+        <v>1.2</v>
       </c>
       <c r="E2">
-        <v>2.4</v>
+        <v>4.2</v>
       </c>
       <c r="F2" s="1">
-        <v>564.55</v>
+        <v>765.11</v>
       </c>
       <c r="G2" s="1">
-        <v>235.2291666666667</v>
+        <v>182.1690476190476</v>
       </c>
       <c r="H2" s="1">
-        <v>772.7130877469586</v>
+        <v>487.1037412160916</v>
       </c>
       <c r="I2" s="1">
-        <v>349.3005877469586</v>
+        <v>268.5008840732345</v>
       </c>
       <c r="J2" s="1">
-        <v>92.12803001826033</v>
+        <v>70.81710817431559</v>
       </c>
       <c r="K2" s="1">
-        <v>680.5850577286983</v>
+        <v>416.286633041776</v>
       </c>
       <c r="L2" s="2">
-        <v>0.1192266980838684</v>
+        <v>0.1453840366684832</v>
       </c>
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="C3" s="4">
-        <v>45112</v>
+        <v>43651</v>
       </c>
       <c r="D3">
-        <v>7.3</v>
+        <v>3.2</v>
       </c>
       <c r="E3">
-        <v>7.3</v>
+        <v>3.2</v>
       </c>
       <c r="F3" s="1">
-        <v>2291.93</v>
+        <v>611.72</v>
       </c>
       <c r="G3" s="1">
-        <v>313.9630136986301</v>
+        <v>191.1625</v>
       </c>
       <c r="H3" s="1">
-        <v>3133.780855862665</v>
+        <v>1298.943309909578</v>
       </c>
       <c r="I3" s="1">
-        <v>841.8508558626655</v>
+        <v>687.2233099095776</v>
       </c>
       <c r="J3" s="1">
-        <v>222.038163233778</v>
+        <v>181.2551479886511</v>
       </c>
       <c r="K3" s="1">
-        <v>2911.742692628887</v>
+        <v>1117.688161920927</v>
       </c>
       <c r="L3" s="2">
-        <v>0.07085312389294544</v>
+        <v>0.1395404607775136</v>
       </c>
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="C4" s="4">
-        <v>45509</v>
+        <v>44382</v>
       </c>
       <c r="D4">
-        <v>4</v>
+        <v>0.5999999999999996</v>
       </c>
       <c r="E4">
-        <v>4</v>
+        <v>2.4</v>
       </c>
       <c r="F4" s="1">
-        <v>1509.1</v>
+        <v>564.55</v>
       </c>
       <c r="G4" s="1">
-        <v>377.275</v>
+        <v>235.2291666666667</v>
       </c>
       <c r="H4" s="1">
-        <v>1717.140194993241</v>
+        <v>243.5518706080456</v>
       </c>
       <c r="I4" s="1">
-        <v>208.0401949932414</v>
+        <v>102.4143706080457</v>
       </c>
       <c r="J4" s="1">
-        <v>54.87060142946741</v>
+        <v>27.01179024787206</v>
       </c>
       <c r="K4" s="1">
-        <v>1662.269593563774</v>
+        <v>216.5400803601736</v>
       </c>
       <c r="L4" s="2">
-        <v>0.0319546427190142</v>
+        <v>0.1109077511104106</v>
       </c>
     </row>
   </sheetData>
@@ -635,20 +1048,114 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="14.28515625" customWidth="1"/>
+    <col min="2" max="2" width="26.28515625" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="4" max="5" width="12.7109375" customWidth="1"/>
+    <col min="6" max="11" width="15.7109375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="15.7109375" style="2" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="50" customHeight="1">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="4">
+        <v>44272</v>
+      </c>
+      <c r="D2">
+        <v>10</v>
+      </c>
+      <c r="E2">
+        <v>10</v>
+      </c>
+      <c r="F2" s="1">
+        <v>352.4</v>
+      </c>
+      <c r="G2" s="1">
+        <v>35.23999999999999</v>
+      </c>
+      <c r="H2" s="1">
+        <v>860.1</v>
+      </c>
+      <c r="I2" s="1">
+        <v>507.7000000000001</v>
+      </c>
+      <c r="J2" s="1">
+        <v>133.905875</v>
+      </c>
+      <c r="K2" s="1">
+        <v>726.194125</v>
+      </c>
+      <c r="L2" s="2">
+        <v>0.155686402743867</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.28515625" customWidth="1"/>
     <col min="2" max="2" width="38.28515625" customWidth="1"/>
     <col min="3" max="3" width="12.28515625" customWidth="1"/>
     <col min="4" max="5" width="12.7109375" customWidth="1"/>
-    <col min="6" max="14" width="15.7109375" style="1" customWidth="1"/>
-    <col min="15" max="15" width="15.7109375" style="2" customWidth="1"/>
+    <col min="6" max="11" width="15.7109375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="15.7109375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="50" customHeight="1">
+    <row r="1" spans="1:12" ht="50" customHeight="1">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -656,51 +1163,42 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
+      <c r="I1" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="K1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="3" t="s">
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
         <v>17</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15">
-      <c r="A2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" t="s">
-        <v>25</v>
       </c>
       <c r="C2" s="4">
         <v>45691</v>
@@ -718,28 +1216,19 @@
         <v>26.185</v>
       </c>
       <c r="H2" s="1">
-        <v>0.4147</v>
+        <v>617.1</v>
       </c>
       <c r="I2" s="1">
-        <v>0.4147</v>
+        <v>65.37999999999997</v>
       </c>
       <c r="J2" s="1">
-        <v>26.5997</v>
+        <v>17.24397499999999</v>
       </c>
       <c r="K2" s="1">
-        <v>480.3</v>
-      </c>
-      <c r="L2" s="1">
-        <v>-36.18580000000002</v>
-      </c>
-      <c r="M2" s="1">
-        <v>0</v>
-      </c>
-      <c r="N2" s="1">
-        <v>480.3</v>
-      </c>
-      <c r="O2" s="2">
-        <v>0</v>
+        <v>599.856025</v>
+      </c>
+      <c r="L2" s="2">
+        <v>0.02794356668287148</v>
       </c>
     </row>
   </sheetData>
@@ -748,6 +1237,495 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="14.28515625" customWidth="1"/>
+    <col min="2" max="2" width="38.28515625" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="4" max="11" width="15.7109375" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="50" customHeight="1">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="1">
+        <v>0</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0</v>
+      </c>
+      <c r="G2" s="1">
+        <v>0</v>
+      </c>
+      <c r="H2" s="1">
+        <v>8.895079561666668</v>
+      </c>
+      <c r="I2" s="1">
+        <v>6.226555693166667</v>
+      </c>
+      <c r="J2" s="1">
+        <v>8.895079561666668</v>
+      </c>
+      <c r="K2" s="1">
+        <v>6.226555693166667</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" s="1">
+        <v>84.53851220416665</v>
+      </c>
+      <c r="E3" s="1">
+        <v>59.17695854291665</v>
+      </c>
+      <c r="F3" s="1">
+        <v>105.8680523496667</v>
+      </c>
+      <c r="G3" s="1">
+        <v>74.10763664476667</v>
+      </c>
+      <c r="H3" s="1">
+        <v>170.6344257453333</v>
+      </c>
+      <c r="I3" s="1">
+        <v>119.4440980217333</v>
+      </c>
+      <c r="J3" s="1">
+        <v>361.0409902991667</v>
+      </c>
+      <c r="K3" s="1">
+        <v>252.7286932094167</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="1">
+        <v>84.53851220416665</v>
+      </c>
+      <c r="E4" s="1">
+        <v>59.17695854291665</v>
+      </c>
+      <c r="F4" s="1">
+        <v>105.8680523496667</v>
+      </c>
+      <c r="G4" s="1">
+        <v>74.10763664476667</v>
+      </c>
+      <c r="H4" s="1">
+        <v>179.529505307</v>
+      </c>
+      <c r="I4" s="1">
+        <v>125.6706537149</v>
+      </c>
+      <c r="J4" s="1">
+        <v>369.9360698608334</v>
+      </c>
+      <c r="K4" s="1">
+        <v>258.9552489025833</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="1">
+        <v>9.625587516666666</v>
+      </c>
+      <c r="E6" s="1">
+        <v>6.737911261666666</v>
+      </c>
+      <c r="F6" s="1">
+        <v>15.5869336875</v>
+      </c>
+      <c r="G6" s="1">
+        <v>10.91085358125</v>
+      </c>
+      <c r="H6" s="1">
+        <v>0</v>
+      </c>
+      <c r="I6" s="1">
+        <v>0</v>
+      </c>
+      <c r="J6" s="1">
+        <v>25.21252120416667</v>
+      </c>
+      <c r="K6" s="1">
+        <v>17.64876484291666</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="1">
+        <v>0</v>
+      </c>
+      <c r="E7" s="1">
+        <v>0</v>
+      </c>
+      <c r="F7" s="1">
+        <v>0</v>
+      </c>
+      <c r="G7" s="1">
+        <v>0</v>
+      </c>
+      <c r="H7" s="1">
+        <v>47.00843371</v>
+      </c>
+      <c r="I7" s="1">
+        <v>32.905903597</v>
+      </c>
+      <c r="J7" s="1">
+        <v>47.00843371</v>
+      </c>
+      <c r="K7" s="1">
+        <v>32.905903597</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" s="1">
+        <v>8.18907125</v>
+      </c>
+      <c r="E8" s="1">
+        <v>5.732349875</v>
+      </c>
+      <c r="F8" s="1">
+        <v>8.5908617</v>
+      </c>
+      <c r="G8" s="1">
+        <v>6.01360319</v>
+      </c>
+      <c r="H8" s="1">
+        <v>11.9130388</v>
+      </c>
+      <c r="I8" s="1">
+        <v>8.339127159999999</v>
+      </c>
+      <c r="J8" s="1">
+        <v>28.69297175</v>
+      </c>
+      <c r="K8" s="1">
+        <v>20.085080225</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="1">
+        <v>17.81465876666667</v>
+      </c>
+      <c r="E9" s="1">
+        <v>12.47026113666666</v>
+      </c>
+      <c r="F9" s="1">
+        <v>24.1777953875</v>
+      </c>
+      <c r="G9" s="1">
+        <v>16.92445677125</v>
+      </c>
+      <c r="H9" s="1">
+        <v>58.92147251</v>
+      </c>
+      <c r="I9" s="1">
+        <v>41.24503075699999</v>
+      </c>
+      <c r="J9" s="1">
+        <v>100.9139266641667</v>
+      </c>
+      <c r="K9" s="1">
+        <v>70.63974866491665</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" s="1">
+        <v>102.3531709708333</v>
+      </c>
+      <c r="E11" s="1">
+        <v>71.64721967958332</v>
+      </c>
+      <c r="F11" s="1">
+        <v>130.0458477371667</v>
+      </c>
+      <c r="G11" s="1">
+        <v>91.03209341601666</v>
+      </c>
+      <c r="H11" s="1">
+        <v>238.450977817</v>
+      </c>
+      <c r="I11" s="1">
+        <v>166.9156844719</v>
+      </c>
+      <c r="J11" s="1">
+        <v>470.8499965250001</v>
+      </c>
+      <c r="K11" s="1">
+        <v>329.5949975675</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="14.28515625" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="4" max="5" width="12.7109375" customWidth="1"/>
+    <col min="6" max="11" width="15.7109375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="15.7109375" style="2" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="50" customHeight="1">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="4">
+        <v>44382</v>
+      </c>
+      <c r="D2">
+        <v>1.8</v>
+      </c>
+      <c r="E2">
+        <v>2.4</v>
+      </c>
+      <c r="F2" s="1">
+        <v>564.55</v>
+      </c>
+      <c r="G2" s="1">
+        <v>235.2291666666667</v>
+      </c>
+      <c r="H2" s="1">
+        <v>730.6556118241375</v>
+      </c>
+      <c r="I2" s="1">
+        <v>307.2431118241374</v>
+      </c>
+      <c r="J2" s="1">
+        <v>81.03537074361624</v>
+      </c>
+      <c r="K2" s="1">
+        <v>649.6202410805213</v>
+      </c>
+      <c r="L2" s="2">
+        <v>0.1109077511104106</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="4">
+        <v>45112</v>
+      </c>
+      <c r="D3">
+        <v>7.3</v>
+      </c>
+      <c r="E3">
+        <v>7.3</v>
+      </c>
+      <c r="F3" s="1">
+        <v>2291.93</v>
+      </c>
+      <c r="G3" s="1">
+        <v>313.9630136986301</v>
+      </c>
+      <c r="H3" s="1">
+        <v>2963.214425731223</v>
+      </c>
+      <c r="I3" s="1">
+        <v>671.2844257312239</v>
+      </c>
+      <c r="J3" s="1">
+        <v>177.0512672866103</v>
+      </c>
+      <c r="K3" s="1">
+        <v>2786.163158444613</v>
+      </c>
+      <c r="L3" s="2">
+        <v>0.05974973182810416</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="4">
+        <v>45509</v>
+      </c>
+      <c r="D4">
+        <v>4</v>
+      </c>
+      <c r="E4">
+        <v>4</v>
+      </c>
+      <c r="F4" s="1">
+        <v>1509.1</v>
+      </c>
+      <c r="G4" s="1">
+        <v>377.275</v>
+      </c>
+      <c r="H4" s="1">
+        <v>1623.679137386972</v>
+      </c>
+      <c r="I4" s="1">
+        <v>114.579137386972</v>
+      </c>
+      <c r="J4" s="1">
+        <v>30.22024748581386</v>
+      </c>
+      <c r="K4" s="1">
+        <v>1593.458889901158</v>
+      </c>
+      <c r="L4" s="2">
+        <v>0.01861220409252044</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:O3"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -768,51 +1746,51 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="K1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
+      <c r="L1" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="N1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="K1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:15">
       <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
         <v>18</v>
-      </c>
-      <c r="B2" t="s">
-        <v>19</v>
       </c>
       <c r="C2" s="4">
         <v>43816</v>
@@ -830,36 +1808,36 @@
         <v>82.84</v>
       </c>
       <c r="H2" s="1">
-        <v>0.39021</v>
+        <v>0.35344687</v>
       </c>
       <c r="I2" s="1">
-        <v>0.39021</v>
+        <v>0.35344687</v>
       </c>
       <c r="J2" s="1">
-        <v>83.23021</v>
+        <v>83.19344687</v>
       </c>
       <c r="K2" s="1">
-        <v>1389.8</v>
+        <v>1605</v>
       </c>
       <c r="L2" s="1">
-        <v>390.2485299999999</v>
+        <v>541.14587191</v>
       </c>
       <c r="M2" s="1">
-        <v>102.9280497875</v>
+        <v>142.7272237162625</v>
       </c>
       <c r="N2" s="1">
-        <v>1286.8719502125</v>
+        <v>1462.272776283738</v>
       </c>
       <c r="O2" s="2">
-        <v>0.07405961274104186</v>
+        <v>0.08892661913785825</v>
       </c>
     </row>
     <row r="3" spans="1:15">
       <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
         <v>18</v>
-      </c>
-      <c r="B3" t="s">
-        <v>19</v>
       </c>
       <c r="C3" s="4">
         <v>43819</v>
@@ -877,28 +1855,28 @@
         <v>83.98</v>
       </c>
       <c r="H3" s="1">
-        <v>0.39021</v>
+        <v>0.35344687</v>
       </c>
       <c r="I3" s="1">
-        <v>0.39021</v>
+        <v>0.35344687</v>
       </c>
       <c r="J3" s="1">
-        <v>84.37021</v>
+        <v>84.33344687</v>
       </c>
       <c r="K3" s="1">
-        <v>17094.54</v>
+        <v>19741.5</v>
       </c>
       <c r="L3" s="1">
-        <v>4701.902918999999</v>
+        <v>6557.940224492999</v>
       </c>
       <c r="M3" s="1">
-        <v>1240.12689488625</v>
+        <v>1729.656734210028</v>
       </c>
       <c r="N3" s="1">
-        <v>15854.41310511375</v>
+        <v>18011.84326578997</v>
       </c>
       <c r="O3" s="2">
-        <v>0.07254520419304936</v>
+        <v>0.08761526399767132</v>
       </c>
     </row>
   </sheetData>
@@ -906,7 +1884,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Q2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -927,57 +1905,57 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="M1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
+      <c r="N1" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="P1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="M1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:17">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C2" s="4">
         <v>43837</v>
@@ -995,34 +1973,34 @@
         <v>78.59</v>
       </c>
       <c r="H2" s="1">
-        <v>1.63781</v>
+        <v>1.63781425</v>
       </c>
       <c r="I2" s="1">
-        <v>1.71817</v>
+        <v>1.71817234</v>
       </c>
       <c r="J2" s="1">
-        <v>2.39935</v>
+        <v>2.38260776</v>
       </c>
       <c r="K2" s="1">
-        <v>5.75533</v>
+        <v>5.73859435</v>
       </c>
       <c r="L2" s="1">
-        <v>84.34533</v>
+        <v>84.32859435</v>
       </c>
       <c r="M2" s="1">
-        <v>709</v>
+        <v>824</v>
       </c>
       <c r="N2" s="1">
-        <v>201.091345</v>
+        <v>281.649919775</v>
       </c>
       <c r="O2" s="1">
-        <v>53.03784224375001</v>
+        <v>74.28516634065625</v>
       </c>
       <c r="P2" s="1">
-        <v>655.96215775625</v>
+        <v>749.7148336593438</v>
       </c>
       <c r="Q2" s="2">
-        <v>0.07480654759344148</v>
+        <v>0.09015190089885466</v>
       </c>
     </row>
   </sheetData>
@@ -1030,20 +2008,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.28515625" customWidth="1"/>
     <col min="2" max="2" width="38.28515625" customWidth="1"/>
     <col min="3" max="3" width="12.28515625" customWidth="1"/>
     <col min="4" max="5" width="12.7109375" customWidth="1"/>
-    <col min="6" max="16" width="15.7109375" style="1" customWidth="1"/>
-    <col min="17" max="17" width="15.7109375" style="2" customWidth="1"/>
+    <col min="6" max="15" width="15.7109375" style="1" customWidth="1"/>
+    <col min="16" max="16" width="15.7109375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="50" customHeight="1">
+    <row r="1" spans="1:16" ht="50" customHeight="1">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1051,57 +2029,54 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
+      <c r="M1" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="O1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="M1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="N1" s="3" t="s">
+    </row>
+    <row r="2" spans="1:16">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
         <v>17</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17">
-      <c r="A2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" t="s">
-        <v>25</v>
       </c>
       <c r="C2" s="4">
         <v>44166</v>
@@ -1119,42 +2094,39 @@
         <v>8.448399999999999</v>
       </c>
       <c r="H2" s="1">
-        <v>0.18936</v>
+        <v>0.18935582</v>
       </c>
       <c r="I2" s="1">
-        <v>0.24135</v>
+        <v>0.24134607</v>
       </c>
       <c r="J2" s="1">
-        <v>0.4524</v>
+        <v>0.43070189</v>
       </c>
       <c r="K2" s="1">
-        <v>0.8831100000000001</v>
+        <v>8.879101889999999</v>
       </c>
       <c r="L2" s="1">
-        <v>9.33151</v>
+        <v>1542.75</v>
       </c>
       <c r="M2" s="1">
-        <v>1200.75</v>
+        <v>769.15643385</v>
       </c>
       <c r="N2" s="1">
-        <v>513.92215</v>
+        <v>202.8650094279375</v>
       </c>
       <c r="O2" s="1">
-        <v>135.5469670625</v>
-      </c>
-      <c r="P2" s="1">
-        <v>1065.2030329375</v>
-      </c>
-      <c r="Q2" s="2">
-        <v>0.1128852526025401</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17">
+        <v>1339.884990572063</v>
+      </c>
+      <c r="P2" s="2">
+        <v>0.1314957118314292</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="C3" s="4">
         <v>45261</v>
@@ -1172,42 +2144,39 @@
         <v>14.345</v>
       </c>
       <c r="H3" s="1">
-        <v>0.01578</v>
+        <v>0.01577965166666667</v>
       </c>
       <c r="I3" s="1">
-        <v>0.24135</v>
+        <v>0.24134607</v>
       </c>
       <c r="J3" s="1">
-        <v>0.4524</v>
+        <v>0.2571257216666666</v>
       </c>
       <c r="K3" s="1">
-        <v>0.70953</v>
+        <v>14.60212572166667</v>
       </c>
       <c r="L3" s="1">
-        <v>15.05453</v>
+        <v>308.55</v>
       </c>
       <c r="M3" s="1">
-        <v>240.15</v>
+        <v>113.7701199483334</v>
       </c>
       <c r="N3" s="1">
-        <v>62.72329000000001</v>
+        <v>30.00686913637292</v>
       </c>
       <c r="O3" s="1">
-        <v>16.5432677375</v>
-      </c>
-      <c r="P3" s="1">
-        <v>223.6067322625</v>
-      </c>
-      <c r="Q3" s="2">
-        <v>0.06888722772225692</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17">
+        <v>278.5431308636271</v>
+      </c>
+      <c r="P3" s="2">
+        <v>0.09725123687043565</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="C4" s="4">
         <v>45627</v>
@@ -1225,31 +2194,28 @@
         <v>25.35327272727273</v>
       </c>
       <c r="I4" s="1">
-        <v>0.0201125</v>
+        <v>0.0201121725</v>
       </c>
       <c r="J4" s="1">
-        <v>0.4524</v>
+        <v>0.0201121725</v>
       </c>
       <c r="K4" s="1">
-        <v>0.4725125</v>
+        <v>25.37338489977273</v>
       </c>
       <c r="L4" s="1">
-        <v>25.82578522727273</v>
+        <v>1697.025</v>
       </c>
       <c r="M4" s="1">
-        <v>1320.825</v>
+        <v>211.04218135875</v>
       </c>
       <c r="N4" s="1">
-        <v>-69.71523125000002</v>
+        <v>55.66237533337031</v>
       </c>
       <c r="O4" s="1">
-        <v>-18.3873922421875</v>
-      </c>
-      <c r="P4" s="1">
-        <v>1339.212392242187</v>
-      </c>
-      <c r="Q4" s="2">
-        <v>-0.01392114189403403</v>
+        <v>1641.36262466663</v>
+      </c>
+      <c r="P4" s="2">
+        <v>0.03279997367945098</v>
       </c>
     </row>
   </sheetData>
@@ -1257,7 +2223,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Q16"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1278,57 +2244,57 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="M1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
+      <c r="N1" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="P1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="M1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:17">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C2" s="4">
         <v>43588</v>
@@ -1346,42 +2312,42 @@
         <v>71.84927536231883</v>
       </c>
       <c r="H2" s="1">
-        <v>1.63781</v>
+        <v>1.63781425</v>
       </c>
       <c r="I2" s="1">
-        <v>1.71817</v>
+        <v>1.71817234</v>
       </c>
       <c r="J2" s="1">
-        <v>2.39935</v>
+        <v>2.38260776</v>
       </c>
       <c r="K2" s="1">
-        <v>5.75533</v>
+        <v>5.73859435</v>
       </c>
       <c r="L2" s="1">
-        <v>77.60460536231884</v>
+        <v>77.58786971231883</v>
       </c>
       <c r="M2" s="1">
-        <v>205.61</v>
+        <v>238.96</v>
       </c>
       <c r="N2" s="1">
-        <v>65.1583255572464</v>
+        <v>88.52031224199642</v>
       </c>
       <c r="O2" s="1">
-        <v>17.18550836572374</v>
+        <v>23.34723235382656</v>
       </c>
       <c r="P2" s="1">
-        <v>188.4244916342763</v>
+        <v>215.6127676461735</v>
       </c>
       <c r="Q2" s="2">
-        <v>0.08358303762328552</v>
+        <v>0.09770351671336856</v>
       </c>
     </row>
     <row r="3" spans="1:17">
       <c r="A3" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C3" s="4">
         <v>43772</v>
@@ -1399,42 +2365,42 @@
         <v>73.30010834236185</v>
       </c>
       <c r="H3" s="1">
-        <v>1.63781</v>
+        <v>1.63781425</v>
       </c>
       <c r="I3" s="1">
-        <v>1.71817</v>
+        <v>1.71817234</v>
       </c>
       <c r="J3" s="1">
-        <v>2.39935</v>
+        <v>2.38260776</v>
       </c>
       <c r="K3" s="1">
-        <v>5.75533</v>
+        <v>5.73859435</v>
       </c>
       <c r="L3" s="1">
-        <v>79.05543834236185</v>
+        <v>79.03870269236185</v>
       </c>
       <c r="M3" s="1">
-        <v>1308.814</v>
+        <v>1521.104</v>
       </c>
       <c r="N3" s="1">
-        <v>405.3926128700002</v>
+        <v>554.1037419046502</v>
       </c>
       <c r="O3" s="1">
-        <v>106.9223016444626</v>
+        <v>146.1448619273515</v>
       </c>
       <c r="P3" s="1">
-        <v>1201.891698355538</v>
+        <v>1374.959138072649</v>
       </c>
       <c r="Q3" s="2">
-        <v>0.08169403875910751</v>
+        <v>0.09607815239940955</v>
       </c>
     </row>
     <row r="4" spans="1:17">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C4" s="4">
         <v>43833</v>
@@ -1452,42 +2418,42 @@
         <v>77.52898550724638</v>
       </c>
       <c r="H4" s="1">
-        <v>1.63781</v>
+        <v>1.63781425</v>
       </c>
       <c r="I4" s="1">
-        <v>1.71817</v>
+        <v>1.71817234</v>
       </c>
       <c r="J4" s="1">
-        <v>2.39935</v>
+        <v>2.38260776</v>
       </c>
       <c r="K4" s="1">
-        <v>5.75533</v>
+        <v>5.73859435</v>
       </c>
       <c r="L4" s="1">
-        <v>83.28431550724638</v>
+        <v>83.26757985724637</v>
       </c>
       <c r="M4" s="1">
-        <v>782.736</v>
+        <v>909.696</v>
       </c>
       <c r="N4" s="1">
-        <v>226.10460488</v>
+        <v>315.0412714316</v>
       </c>
       <c r="O4" s="1">
-        <v>59.6350895371</v>
+        <v>83.0921353400845</v>
       </c>
       <c r="P4" s="1">
-        <v>723.1009104628999</v>
+        <v>826.6038646599155</v>
       </c>
       <c r="Q4" s="2">
-        <v>0.07618799893846712</v>
+        <v>0.09134055260228087</v>
       </c>
     </row>
     <row r="5" spans="1:17">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C5" s="4">
         <v>43893</v>
@@ -1505,42 +2471,42 @@
         <v>72.01000000000001</v>
       </c>
       <c r="H5" s="1">
-        <v>1.63781</v>
+        <v>1.63781425</v>
       </c>
       <c r="I5" s="1">
-        <v>1.71817</v>
+        <v>1.71817234</v>
       </c>
       <c r="J5" s="1">
-        <v>2.39935</v>
+        <v>2.38260776</v>
       </c>
       <c r="K5" s="1">
-        <v>5.75533</v>
+        <v>5.73859435</v>
       </c>
       <c r="L5" s="1">
-        <v>77.76533000000001</v>
+        <v>77.74859435</v>
       </c>
       <c r="M5" s="1">
-        <v>709</v>
+        <v>824</v>
       </c>
       <c r="N5" s="1">
-        <v>224.121345</v>
+        <v>304.679919775</v>
       </c>
       <c r="O5" s="1">
-        <v>59.11200474374999</v>
+        <v>80.35932884065625</v>
       </c>
       <c r="P5" s="1">
-        <v>649.88799525625</v>
+        <v>743.6406711593438</v>
       </c>
       <c r="Q5" s="2">
-        <v>0.08337377255818053</v>
+        <v>0.0975234573308935</v>
       </c>
     </row>
     <row r="6" spans="1:17">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C6" s="4">
         <v>44168</v>
@@ -1558,42 +2524,42 @@
         <v>80.2</v>
       </c>
       <c r="H6" s="1">
-        <v>1.63781</v>
+        <v>1.63781425</v>
       </c>
       <c r="I6" s="1">
-        <v>1.71817</v>
+        <v>1.71817234</v>
       </c>
       <c r="J6" s="1">
-        <v>2.39935</v>
+        <v>2.38260776</v>
       </c>
       <c r="K6" s="1">
-        <v>5.75533</v>
+        <v>5.73859435</v>
       </c>
       <c r="L6" s="1">
-        <v>85.95533</v>
+        <v>85.93859435</v>
       </c>
       <c r="M6" s="1">
-        <v>709</v>
+        <v>824</v>
       </c>
       <c r="N6" s="1">
-        <v>195.456345</v>
+        <v>276.014919775</v>
       </c>
       <c r="O6" s="1">
-        <v>51.55161099375</v>
+        <v>72.79893509065624</v>
       </c>
       <c r="P6" s="1">
-        <v>657.44838900625</v>
+        <v>751.2010649093438</v>
       </c>
       <c r="Q6" s="2">
-        <v>0.07271031169781382</v>
+        <v>0.08834822219739835</v>
       </c>
     </row>
     <row r="7" spans="1:17">
       <c r="A7" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C7" s="4">
         <v>44199</v>
@@ -1611,42 +2577,42 @@
         <v>81.42</v>
       </c>
       <c r="H7" s="1">
-        <v>1.63781</v>
+        <v>1.63781425</v>
       </c>
       <c r="I7" s="1">
-        <v>1.71817</v>
+        <v>1.71817234</v>
       </c>
       <c r="J7" s="1">
-        <v>2.39935</v>
+        <v>2.38260776</v>
       </c>
       <c r="K7" s="1">
-        <v>5.75533</v>
+        <v>5.73859435</v>
       </c>
       <c r="L7" s="1">
-        <v>87.17533</v>
+        <v>87.15859435</v>
       </c>
       <c r="M7" s="1">
-        <v>709</v>
+        <v>824</v>
       </c>
       <c r="N7" s="1">
-        <v>191.186345</v>
+        <v>271.744919775</v>
       </c>
       <c r="O7" s="1">
-        <v>50.42539849375001</v>
+        <v>71.67272259065625</v>
       </c>
       <c r="P7" s="1">
-        <v>658.57460150625</v>
+        <v>752.3272774093438</v>
       </c>
       <c r="Q7" s="2">
-        <v>0.07112185965267985</v>
+        <v>0.08698145945467992</v>
       </c>
     </row>
     <row r="8" spans="1:17">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C8" s="4">
         <v>44533</v>
@@ -1664,42 +2630,42 @@
         <v>100.18</v>
       </c>
       <c r="H8" s="1">
-        <v>1.63781</v>
+        <v>1.63781425</v>
       </c>
       <c r="I8" s="1">
-        <v>1.71817</v>
+        <v>1.71817234</v>
       </c>
       <c r="J8" s="1">
-        <v>2.39935</v>
+        <v>2.38260776</v>
       </c>
       <c r="K8" s="1">
-        <v>5.75533</v>
+        <v>5.73859435</v>
       </c>
       <c r="L8" s="1">
-        <v>105.93533</v>
+        <v>105.91859435</v>
       </c>
       <c r="M8" s="1">
-        <v>709</v>
+        <v>824</v>
       </c>
       <c r="N8" s="1">
-        <v>125.526345</v>
+        <v>206.0849197750001</v>
       </c>
       <c r="O8" s="1">
-        <v>33.10757349375001</v>
+        <v>54.35489759065627</v>
       </c>
       <c r="P8" s="1">
-        <v>675.89242650625</v>
+        <v>769.6451024093437</v>
       </c>
       <c r="Q8" s="2">
-        <v>0.04669615443406207</v>
+        <v>0.06596468154205858</v>
       </c>
     </row>
     <row r="9" spans="1:17">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C9" s="4">
         <v>44564</v>
@@ -1717,42 +2683,42 @@
         <v>104.8</v>
       </c>
       <c r="H9" s="1">
-        <v>1.63781</v>
+        <v>1.63781425</v>
       </c>
       <c r="I9" s="1">
-        <v>1.71817</v>
+        <v>1.71817234</v>
       </c>
       <c r="J9" s="1">
-        <v>2.39935</v>
+        <v>2.38260776</v>
       </c>
       <c r="K9" s="1">
-        <v>5.75533</v>
+        <v>5.73859435</v>
       </c>
       <c r="L9" s="1">
-        <v>110.55533</v>
+        <v>110.53859435</v>
       </c>
       <c r="M9" s="1">
-        <v>709</v>
+        <v>824</v>
       </c>
       <c r="N9" s="1">
-        <v>109.3563450000001</v>
+        <v>189.914919775</v>
       </c>
       <c r="O9" s="1">
-        <v>28.84273599375001</v>
+        <v>50.09006009065626</v>
       </c>
       <c r="P9" s="1">
-        <v>680.15726400625</v>
+        <v>773.9099399093437</v>
       </c>
       <c r="Q9" s="2">
-        <v>0.04068086882052188</v>
+        <v>0.06078890787701002</v>
       </c>
     </row>
     <row r="10" spans="1:17">
       <c r="A10" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C10" s="4">
         <v>44898</v>
@@ -1770,42 +2736,42 @@
         <v>96.17999999999999</v>
       </c>
       <c r="H10" s="1">
-        <v>1.63781</v>
+        <v>1.63781425</v>
       </c>
       <c r="I10" s="1">
-        <v>1.71817</v>
+        <v>1.71817234</v>
       </c>
       <c r="J10" s="1">
-        <v>2.39935</v>
+        <v>2.38260776</v>
       </c>
       <c r="K10" s="1">
-        <v>5.75533</v>
+        <v>5.73859435</v>
       </c>
       <c r="L10" s="1">
-        <v>101.93533</v>
+        <v>101.91859435</v>
       </c>
       <c r="M10" s="1">
-        <v>709</v>
+        <v>824</v>
       </c>
       <c r="N10" s="1">
-        <v>139.526345</v>
+        <v>220.0849197750001</v>
       </c>
       <c r="O10" s="1">
-        <v>36.80007349375001</v>
+        <v>58.04739759065627</v>
       </c>
       <c r="P10" s="1">
-        <v>672.19992650625</v>
+        <v>765.9526024093437</v>
       </c>
       <c r="Q10" s="2">
-        <v>0.05190419392630467</v>
+        <v>0.07044587086244693</v>
       </c>
     </row>
     <row r="11" spans="1:17">
       <c r="A11" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C11" s="4">
         <v>44929</v>
@@ -1823,42 +2789,42 @@
         <v>91.65000000000001</v>
       </c>
       <c r="H11" s="1">
-        <v>1.63781</v>
+        <v>1.63781425</v>
       </c>
       <c r="I11" s="1">
-        <v>1.71817</v>
+        <v>1.71817234</v>
       </c>
       <c r="J11" s="1">
-        <v>2.39935</v>
+        <v>2.38260776</v>
       </c>
       <c r="K11" s="1">
-        <v>5.75533</v>
+        <v>5.73859435</v>
       </c>
       <c r="L11" s="1">
-        <v>97.40533000000001</v>
+        <v>97.38859435000001</v>
       </c>
       <c r="M11" s="1">
-        <v>709</v>
+        <v>824</v>
       </c>
       <c r="N11" s="1">
-        <v>155.381345</v>
+        <v>235.939919775</v>
       </c>
       <c r="O11" s="1">
-        <v>40.98182974375</v>
+        <v>62.22915384065625</v>
       </c>
       <c r="P11" s="1">
-        <v>668.01817025625</v>
+        <v>761.7708461593437</v>
       </c>
       <c r="Q11" s="2">
-        <v>0.05780229865126939</v>
+        <v>0.07552081776778671</v>
       </c>
     </row>
     <row r="12" spans="1:17">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C12" s="4">
         <v>45263</v>
@@ -1876,42 +2842,42 @@
         <v>104.12</v>
       </c>
       <c r="H12" s="1">
-        <v>0.1364841666666667</v>
+        <v>0.1364845208333333</v>
       </c>
       <c r="I12" s="1">
-        <v>1.71817</v>
+        <v>1.71817234</v>
       </c>
       <c r="J12" s="1">
-        <v>2.39935</v>
+        <v>2.38260776</v>
       </c>
       <c r="K12" s="1">
-        <v>4.254004166666666</v>
+        <v>4.237264620833333</v>
       </c>
       <c r="L12" s="1">
-        <v>108.3740041666667</v>
+        <v>108.3572646208333</v>
       </c>
       <c r="M12" s="1">
-        <v>709</v>
+        <v>824</v>
       </c>
       <c r="N12" s="1">
-        <v>116.9909854166667</v>
+        <v>197.5495738270834</v>
       </c>
       <c r="O12" s="1">
-        <v>30.85637240364584</v>
+        <v>52.10370009689323</v>
       </c>
       <c r="P12" s="1">
-        <v>678.1436275963541</v>
+        <v>771.8962999031068</v>
       </c>
       <c r="Q12" s="2">
-        <v>0.04352097659188412</v>
+        <v>0.06323264574865683</v>
       </c>
     </row>
     <row r="13" spans="1:17">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C13" s="4">
         <v>45294</v>
@@ -1929,39 +2895,39 @@
         <v>106.62</v>
       </c>
       <c r="I13" s="1">
-        <v>1.71817</v>
+        <v>1.71817234</v>
       </c>
       <c r="J13" s="1">
-        <v>2.39935</v>
+        <v>2.38260776</v>
       </c>
       <c r="K13" s="1">
-        <v>4.11752</v>
+        <v>4.1007801</v>
       </c>
       <c r="L13" s="1">
-        <v>110.73752</v>
+        <v>110.7207801</v>
       </c>
       <c r="M13" s="1">
-        <v>709</v>
+        <v>824</v>
       </c>
       <c r="N13" s="1">
-        <v>108.71868</v>
+        <v>189.27726965</v>
       </c>
       <c r="O13" s="1">
-        <v>28.67455185</v>
+        <v>49.9218798701875</v>
       </c>
       <c r="P13" s="1">
-        <v>680.3254481499999</v>
+        <v>774.0781201298125</v>
       </c>
       <c r="Q13" s="2">
-        <v>0.04044365564174895</v>
+        <v>0.06058480566770328</v>
       </c>
     </row>
     <row r="14" spans="1:17">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B14" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C14" s="4">
         <v>45629</v>
@@ -1979,39 +2945,39 @@
         <v>135.64</v>
       </c>
       <c r="I14" s="1">
-        <v>0.1431808333333333</v>
+        <v>0.1431810283333333</v>
       </c>
       <c r="J14" s="1">
-        <v>2.39935</v>
+        <v>2.38260776</v>
       </c>
       <c r="K14" s="1">
-        <v>2.542530833333333</v>
+        <v>2.525788788333333</v>
       </c>
       <c r="L14" s="1">
-        <v>138.1825308333333</v>
+        <v>138.1657887883333</v>
       </c>
       <c r="M14" s="1">
-        <v>709</v>
+        <v>824</v>
       </c>
       <c r="N14" s="1">
-        <v>12.66114208333333</v>
+        <v>93.21973924083333</v>
       </c>
       <c r="O14" s="1">
-        <v>3.339376224479166</v>
+        <v>24.58670622476979</v>
       </c>
       <c r="P14" s="1">
-        <v>705.6606237755209</v>
+        <v>799.4132937752302</v>
       </c>
       <c r="Q14" s="2">
-        <v>0.004709980570492477</v>
+        <v>0.02983823570967208</v>
       </c>
     </row>
     <row r="15" spans="1:17">
       <c r="A15" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B15" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C15" s="4">
         <v>45660</v>
@@ -2029,36 +2995,36 @@
         <v>135.24</v>
       </c>
       <c r="J15" s="1">
-        <v>2.39935</v>
+        <v>2.38260776</v>
       </c>
       <c r="K15" s="1">
-        <v>2.39935</v>
+        <v>2.38260776</v>
       </c>
       <c r="L15" s="1">
-        <v>137.63935</v>
+        <v>137.62260776</v>
       </c>
       <c r="M15" s="1">
-        <v>709</v>
+        <v>824</v>
       </c>
       <c r="N15" s="1">
-        <v>14.56227500000001</v>
+        <v>95.12087283999996</v>
       </c>
       <c r="O15" s="1">
-        <v>3.840800031250003</v>
+        <v>25.08813021154999</v>
       </c>
       <c r="P15" s="1">
-        <v>705.15919996875</v>
+        <v>798.91186978845</v>
       </c>
       <c r="Q15" s="2">
-        <v>0.005417207378349793</v>
+        <v>0.03044675996547328</v>
       </c>
     </row>
     <row r="16" spans="1:17">
       <c r="A16" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B16" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C16" s="4">
         <v>45994</v>
@@ -2076,28 +3042,28 @@
         <v>144.18</v>
       </c>
       <c r="J16" s="1">
-        <v>0.1999458333333333</v>
+        <v>0.1985506466666667</v>
       </c>
       <c r="K16" s="1">
-        <v>0.1999458333333333</v>
+        <v>0.1985506466666667</v>
       </c>
       <c r="L16" s="1">
-        <v>144.3799458333334</v>
+        <v>144.3785506466667</v>
       </c>
       <c r="M16" s="1">
-        <v>709</v>
+        <v>824</v>
       </c>
       <c r="N16" s="1">
-        <v>-9.029810416666692</v>
+        <v>71.4750727366667</v>
       </c>
       <c r="O16" s="1">
-        <v>-2.38161249739584</v>
+        <v>18.85155043429584</v>
       </c>
       <c r="P16" s="1">
-        <v>711.3816124973958</v>
+        <v>805.1484495657041</v>
       </c>
       <c r="Q16" s="2">
-        <v>-0.003359114946961692</v>
+        <v>0.02287809518725224</v>
       </c>
     </row>
   </sheetData>
@@ -2105,7 +3071,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:O8"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2126,51 +3092,51 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="K1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
+      <c r="L1" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="N1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="K1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:15">
       <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
         <v>18</v>
-      </c>
-      <c r="B2" t="s">
-        <v>19</v>
       </c>
       <c r="C2" s="4">
         <v>43822</v>
@@ -2188,36 +3154,36 @@
         <v>83.88</v>
       </c>
       <c r="H2" s="1">
-        <v>0.39021</v>
+        <v>0.35344687</v>
       </c>
       <c r="I2" s="1">
-        <v>0.39021</v>
+        <v>0.35344687</v>
       </c>
       <c r="J2" s="1">
-        <v>84.27020999999999</v>
+        <v>84.23344686999999</v>
       </c>
       <c r="K2" s="1">
-        <v>416.9399999999999</v>
+        <v>481.5</v>
       </c>
       <c r="L2" s="1">
-        <v>114.890559</v>
+        <v>160.159761573</v>
       </c>
       <c r="M2" s="1">
-        <v>30.30238493625</v>
+        <v>42.24213711487875</v>
       </c>
       <c r="N2" s="1">
-        <v>386.6376150637499</v>
+        <v>439.2578628851213</v>
       </c>
       <c r="O2" s="2">
-        <v>0.07267804704813642</v>
+        <v>0.08773029515031931</v>
       </c>
     </row>
     <row r="3" spans="1:15">
       <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
         <v>18</v>
-      </c>
-      <c r="B3" t="s">
-        <v>19</v>
       </c>
       <c r="C3" s="4">
         <v>44370</v>
@@ -2235,36 +3201,36 @@
         <v>98.44</v>
       </c>
       <c r="H3" s="1">
-        <v>0.39021</v>
+        <v>0.35344687</v>
       </c>
       <c r="I3" s="1">
-        <v>0.39021</v>
+        <v>0.35344687</v>
       </c>
       <c r="J3" s="1">
-        <v>98.83020999999999</v>
+        <v>98.79344687</v>
       </c>
       <c r="K3" s="1">
-        <v>555.92</v>
+        <v>642</v>
       </c>
       <c r="L3" s="1">
-        <v>112.419412</v>
+        <v>172.778348764</v>
       </c>
       <c r="M3" s="1">
-        <v>29.650619915</v>
+        <v>45.570289486505</v>
       </c>
       <c r="N3" s="1">
-        <v>526.269380085</v>
+        <v>596.429710513495</v>
       </c>
       <c r="O3" s="2">
-        <v>0.05333612734746006</v>
+        <v>0.07098175932477414</v>
       </c>
     </row>
     <row r="4" spans="1:15">
       <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
         <v>18</v>
-      </c>
-      <c r="B4" t="s">
-        <v>19</v>
       </c>
       <c r="C4" s="4">
         <v>44400</v>
@@ -2282,36 +3248,36 @@
         <v>101.68</v>
       </c>
       <c r="H4" s="1">
-        <v>0.39021</v>
+        <v>0.35344687</v>
       </c>
       <c r="I4" s="1">
-        <v>0.39021</v>
+        <v>0.35344687</v>
       </c>
       <c r="J4" s="1">
-        <v>102.07021</v>
+        <v>102.03344687</v>
       </c>
       <c r="K4" s="1">
-        <v>555.92</v>
+        <v>642</v>
       </c>
       <c r="L4" s="1">
-        <v>103.347412</v>
+        <v>163.706348764</v>
       </c>
       <c r="M4" s="1">
-        <v>27.25787991499999</v>
+        <v>43.17754948650499</v>
       </c>
       <c r="N4" s="1">
-        <v>528.662120085</v>
+        <v>598.822450513495</v>
       </c>
       <c r="O4" s="2">
-        <v>0.04903201884263921</v>
+        <v>0.06725474997897975</v>
       </c>
     </row>
     <row r="5" spans="1:15">
       <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
         <v>18</v>
-      </c>
-      <c r="B5" t="s">
-        <v>19</v>
       </c>
       <c r="C5" s="4">
         <v>45108</v>
@@ -2329,36 +3295,36 @@
         <v>103.9085714285714</v>
       </c>
       <c r="H5" s="1">
-        <v>0.39021</v>
+        <v>0.35344687</v>
       </c>
       <c r="I5" s="1">
-        <v>0.39021</v>
+        <v>0.35344687</v>
       </c>
       <c r="J5" s="1">
-        <v>104.2987814285714</v>
+        <v>104.2620182985714</v>
       </c>
       <c r="K5" s="1">
-        <v>972.8599999999999</v>
+        <v>1123.5</v>
       </c>
       <c r="L5" s="1">
-        <v>169.9379709999999</v>
+        <v>275.566110337</v>
       </c>
       <c r="M5" s="1">
-        <v>44.82113985124997</v>
+        <v>72.68056160138374</v>
       </c>
       <c r="N5" s="1">
-        <v>928.0388601487499</v>
+        <v>1050.819438398616</v>
       </c>
       <c r="O5" s="2">
-        <v>0.04607152092927037</v>
+        <v>0.06469119857711059</v>
       </c>
     </row>
     <row r="6" spans="1:15">
       <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
         <v>18</v>
-      </c>
-      <c r="B6" t="s">
-        <v>19</v>
       </c>
       <c r="C6" s="4">
         <v>45413</v>
@@ -2376,36 +3342,36 @@
         <v>116.72</v>
       </c>
       <c r="H6" s="1">
-        <v>0.39021</v>
+        <v>0.35344687</v>
       </c>
       <c r="I6" s="1">
-        <v>0.39021</v>
+        <v>0.35344687</v>
       </c>
       <c r="J6" s="1">
-        <v>117.11021</v>
+        <v>117.07344687</v>
       </c>
       <c r="K6" s="1">
-        <v>277.96</v>
+        <v>321</v>
       </c>
       <c r="L6" s="1">
-        <v>30.61770599999999</v>
+        <v>60.797174382</v>
       </c>
       <c r="M6" s="1">
-        <v>8.075419957499998</v>
+        <v>16.0352547432525</v>
       </c>
       <c r="N6" s="1">
-        <v>269.8845800425</v>
+        <v>304.9647452567475</v>
       </c>
       <c r="O6" s="2">
-        <v>0.02905245343754496</v>
+        <v>0.04995406462072429</v>
       </c>
     </row>
     <row r="7" spans="1:15">
       <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
         <v>18</v>
-      </c>
-      <c r="B7" t="s">
-        <v>19</v>
       </c>
       <c r="C7" s="4">
         <v>45787</v>
@@ -2423,36 +3389,36 @@
         <v>123.48</v>
       </c>
       <c r="H7" s="1">
-        <v>0.26014</v>
+        <v>0.2356312466666667</v>
       </c>
       <c r="I7" s="1">
-        <v>0.26014</v>
+        <v>0.2356312466666667</v>
       </c>
       <c r="J7" s="1">
-        <v>123.74014</v>
+        <v>123.7156312466667</v>
       </c>
       <c r="K7" s="1">
-        <v>555.92</v>
+        <v>642</v>
       </c>
       <c r="L7" s="1">
-        <v>42.67160799999994</v>
+        <v>102.9962325093333</v>
       </c>
       <c r="M7" s="1">
-        <v>11.25463660999998</v>
+        <v>27.16525632433666</v>
       </c>
       <c r="N7" s="1">
-        <v>544.6653633899999</v>
+        <v>614.8347436756634</v>
       </c>
       <c r="O7" s="2">
-        <v>0.02024506513527123</v>
+        <v>0.04231348337124091</v>
       </c>
     </row>
     <row r="8" spans="1:15">
       <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s">
         <v>18</v>
-      </c>
-      <c r="B8" t="s">
-        <v>19</v>
       </c>
       <c r="C8" s="4">
         <v>45940</v>
@@ -2470,28 +3436,28 @@
         <v>137.38</v>
       </c>
       <c r="H8" s="1">
-        <v>0.0975525</v>
+        <v>0.08836171750000001</v>
       </c>
       <c r="I8" s="1">
-        <v>0.0975525</v>
+        <v>0.08836171750000001</v>
       </c>
       <c r="J8" s="1">
-        <v>137.4775525</v>
+        <v>137.4683617175</v>
       </c>
       <c r="K8" s="1">
-        <v>1389.8</v>
+        <v>1605</v>
       </c>
       <c r="L8" s="1">
-        <v>10.51713249999992</v>
+        <v>161.2214679775001</v>
       </c>
       <c r="M8" s="1">
-        <v>2.773893696874977</v>
+        <v>42.52216217906565</v>
       </c>
       <c r="N8" s="1">
-        <v>1387.026106303125</v>
+        <v>1562.477837820934</v>
       </c>
       <c r="O8" s="2">
-        <v>0.001995894155184183</v>
+        <v>0.02649355899007205</v>
       </c>
     </row>
   </sheetData>
@@ -2499,7 +3465,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2519,280 +3485,34 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
+      <c r="J1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="K1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12">
-      <c r="A2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C2" s="4">
-        <v>43725</v>
-      </c>
-      <c r="D2">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="E2">
-        <v>10.3</v>
-      </c>
-      <c r="F2" s="1">
-        <v>513.9400000000001</v>
-      </c>
-      <c r="G2" s="1">
-        <v>49.89708737864078</v>
-      </c>
-      <c r="H2" s="1">
-        <v>1926.845</v>
-      </c>
-      <c r="I2" s="1">
-        <v>1512.699174757282</v>
-      </c>
-      <c r="J2" s="1">
-        <v>398.9744073422331</v>
-      </c>
-      <c r="K2" s="1">
-        <v>1527.870592657767</v>
-      </c>
-      <c r="L2" s="2">
-        <v>0.2070609765405277</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
-      <c r="A3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C3" s="4">
-        <v>44609</v>
-      </c>
-      <c r="D3">
-        <v>5</v>
-      </c>
-      <c r="E3">
-        <v>5</v>
-      </c>
-      <c r="F3" s="1">
-        <v>754.7</v>
-      </c>
-      <c r="G3" s="1">
-        <v>150.94</v>
-      </c>
-      <c r="H3" s="1">
-        <v>1160.75</v>
-      </c>
-      <c r="I3" s="1">
-        <v>406.0500000000001</v>
-      </c>
-      <c r="J3" s="1">
-        <v>107.0956875</v>
-      </c>
-      <c r="K3" s="1">
-        <v>1053.6543125</v>
-      </c>
-      <c r="L3" s="2">
-        <v>0.0922642149472324</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12">
-      <c r="A4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" s="4">
-        <v>45124</v>
-      </c>
-      <c r="D4">
-        <v>2</v>
-      </c>
-      <c r="E4">
-        <v>2</v>
-      </c>
-      <c r="F4" s="1">
-        <v>343.52</v>
-      </c>
-      <c r="G4" s="1">
-        <v>171.76</v>
-      </c>
-      <c r="H4" s="1">
-        <v>464.3</v>
-      </c>
-      <c r="I4" s="1">
-        <v>120.78</v>
-      </c>
-      <c r="J4" s="1">
-        <v>31.85572500000001</v>
-      </c>
-      <c r="K4" s="1">
-        <v>432.444275</v>
-      </c>
-      <c r="L4" s="2">
-        <v>0.06861021968554815</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
-      <c r="A5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" s="4">
-        <v>45424</v>
-      </c>
-      <c r="D5">
-        <v>5</v>
-      </c>
-      <c r="E5">
-        <v>5</v>
-      </c>
-      <c r="F5" s="1">
-        <v>847.7</v>
-      </c>
-      <c r="G5" s="1">
-        <v>169.54</v>
-      </c>
-      <c r="H5" s="1">
-        <v>1160.75</v>
-      </c>
-      <c r="I5" s="1">
-        <v>313.05</v>
-      </c>
-      <c r="J5" s="1">
-        <v>82.56693749999998</v>
-      </c>
-      <c r="K5" s="1">
-        <v>1078.1830625</v>
-      </c>
-      <c r="L5" s="2">
-        <v>0.07113240361835019</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
-      <c r="A6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" s="4">
-        <v>46007</v>
-      </c>
-      <c r="D6">
-        <v>4</v>
-      </c>
-      <c r="E6">
-        <v>4</v>
-      </c>
-      <c r="F6" s="1">
-        <v>928.8</v>
-      </c>
-      <c r="G6" s="1">
-        <v>232.2</v>
-      </c>
-      <c r="H6" s="1">
-        <v>928.6</v>
-      </c>
-      <c r="I6" s="1">
-        <v>-0.1999999999999318</v>
-      </c>
-      <c r="J6" s="1">
-        <v>-0.05274999999998201</v>
-      </c>
-      <c r="K6" s="1">
-        <v>928.65275</v>
-      </c>
-      <c r="L6" s="2">
-        <v>-5.680594443245962E-05</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="14.28515625" customWidth="1"/>
-    <col min="2" max="2" width="30.28515625" customWidth="1"/>
-    <col min="3" max="3" width="12.28515625" customWidth="1"/>
-    <col min="4" max="5" width="12.7109375" customWidth="1"/>
-    <col min="6" max="11" width="15.7109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="15.7109375" style="2" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:12" ht="50" customHeight="1">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -2800,37 +3520,37 @@
         <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="C2" s="4">
-        <v>43501</v>
+        <v>43725</v>
       </c>
       <c r="D2">
-        <v>1.2</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="E2">
-        <v>4.2</v>
+        <v>10.3</v>
       </c>
       <c r="F2" s="1">
-        <v>765.11</v>
+        <v>513.9400000000001</v>
       </c>
       <c r="G2" s="1">
-        <v>182.1690476190476</v>
+        <v>49.89708737864078</v>
       </c>
       <c r="H2" s="1">
-        <v>515.1420584979725</v>
+        <v>2245.565000000001</v>
       </c>
       <c r="I2" s="1">
-        <v>296.5392013551153</v>
+        <v>1831.419174757282</v>
       </c>
       <c r="J2" s="1">
-        <v>78.21221435741167</v>
+        <v>483.036807342233</v>
       </c>
       <c r="K2" s="1">
-        <v>436.9298441405608</v>
+        <v>1762.528192657767</v>
       </c>
       <c r="L2" s="2">
-        <v>0.151826497307285</v>
+        <v>0.2151070253331491</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -2838,37 +3558,37 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="C3" s="4">
-        <v>43651</v>
+        <v>44609</v>
       </c>
       <c r="D3">
-        <v>3.2</v>
+        <v>5</v>
       </c>
       <c r="E3">
-        <v>3.2</v>
+        <v>5</v>
       </c>
       <c r="F3" s="1">
-        <v>611.72</v>
+        <v>754.7</v>
       </c>
       <c r="G3" s="1">
-        <v>191.1625</v>
+        <v>150.94</v>
       </c>
       <c r="H3" s="1">
-        <v>1373.712155994593</v>
+        <v>1352.75</v>
       </c>
       <c r="I3" s="1">
-        <v>761.9921559945931</v>
+        <v>598.0500000000001</v>
       </c>
       <c r="J3" s="1">
-        <v>200.9754311435739</v>
+        <v>157.7356875</v>
       </c>
       <c r="K3" s="1">
-        <v>1172.736724851019</v>
+        <v>1195.0143125</v>
       </c>
       <c r="L3" s="2">
-        <v>0.1463009774402586</v>
+        <v>0.1166037238957679</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -2876,131 +3596,113 @@
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="C4" s="4">
-        <v>44382</v>
+        <v>45124</v>
       </c>
       <c r="D4">
-        <v>0.5999999999999996</v>
+        <v>2</v>
       </c>
       <c r="E4">
-        <v>2.4</v>
+        <v>2</v>
       </c>
       <c r="F4" s="1">
-        <v>564.55</v>
+        <v>343.52</v>
       </c>
       <c r="G4" s="1">
-        <v>235.2291666666667</v>
+        <v>171.76</v>
       </c>
       <c r="H4" s="1">
-        <v>257.5710292489861</v>
+        <v>541.1</v>
       </c>
       <c r="I4" s="1">
-        <v>116.4335292489861</v>
+        <v>197.58</v>
       </c>
       <c r="J4" s="1">
-        <v>30.70934333942009</v>
+        <v>52.11172500000001</v>
       </c>
       <c r="K4" s="1">
-        <v>226.861685909566</v>
+        <v>488.988275</v>
       </c>
       <c r="L4" s="2">
-        <v>0.1192266980838684</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="14.28515625" customWidth="1"/>
-    <col min="2" max="2" width="26.28515625" customWidth="1"/>
-    <col min="3" max="3" width="12.28515625" customWidth="1"/>
-    <col min="4" max="5" width="12.7109375" customWidth="1"/>
-    <col min="6" max="11" width="15.7109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="15.7109375" style="2" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:12" ht="50" customHeight="1">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
+        <v>0.09630701349103679</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="4">
+        <v>45424</v>
+      </c>
+      <c r="D5">
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
+      </c>
+      <c r="F5" s="1">
+        <v>847.7</v>
+      </c>
+      <c r="G5" s="1">
+        <v>169.54</v>
+      </c>
+      <c r="H5" s="1">
+        <v>1352.75</v>
+      </c>
+      <c r="I5" s="1">
+        <v>505.05</v>
+      </c>
+      <c r="J5" s="1">
+        <v>133.2069375</v>
+      </c>
+      <c r="K5" s="1">
+        <v>1219.5430625</v>
+      </c>
+      <c r="L5" s="2">
+        <v>0.09847121604139714</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="4">
+        <v>46007</v>
+      </c>
+      <c r="D6">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12">
-      <c r="A2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C2" s="4">
-        <v>44272</v>
-      </c>
-      <c r="D2">
-        <v>10</v>
-      </c>
-      <c r="E2">
-        <v>10</v>
-      </c>
-      <c r="F2" s="1">
-        <v>352.4</v>
-      </c>
-      <c r="G2" s="1">
-        <v>35.23999999999999</v>
-      </c>
-      <c r="H2" s="1">
-        <v>350.95</v>
-      </c>
-      <c r="I2" s="1">
-        <v>-1.44999999999996</v>
-      </c>
-      <c r="J2" s="1">
-        <v>0</v>
-      </c>
-      <c r="K2" s="1">
-        <v>350.95</v>
-      </c>
-      <c r="L2" s="2">
-        <v>0</v>
+      <c r="E6">
+        <v>4</v>
+      </c>
+      <c r="F6" s="1">
+        <v>928.8</v>
+      </c>
+      <c r="G6" s="1">
+        <v>232.2</v>
+      </c>
+      <c r="H6" s="1">
+        <v>1082.2</v>
+      </c>
+      <c r="I6" s="1">
+        <v>153.4000000000001</v>
+      </c>
+      <c r="J6" s="1">
+        <v>40.45925000000002</v>
+      </c>
+      <c r="K6" s="1">
+        <v>1041.74075</v>
+      </c>
+      <c r="L6" s="2">
+        <v>0.03738611162446869</v>
       </c>
     </row>
   </sheetData>

</xml_diff>